<commit_message>
readme, mais primeiro teste para minimax vs aleatorio.
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfbal\Downloads\Projecto2_Alpha4LinhaV3.0\Projecto2_Alpha4'\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfbal\Documents\Projecto2_Alpha4'\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D50092A5-F46C-4E96-BCB7-0047F7D1C1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC0DDCD-6CD4-408E-AE34-DF35A9CEF0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5C53708D-411B-488D-801D-AFAFD207A61B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Comparação</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Humano vs IA (Opcional)</t>
+  </si>
+  <si>
+    <t>O Minimax joga para ganhar e reage ao adversário. O Aleatório joga às cegas, não aproveitando oportunidades nem bloqueando o Minimax, o que explica a taxa de vitórias de 100%.</t>
   </si>
 </sst>
 </file>
@@ -125,8 +128,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,12 +479,12 @@
     <col min="3" max="3" width="15.88671875" customWidth="1"/>
     <col min="4" max="4" width="15.77734375" customWidth="1"/>
     <col min="5" max="5" width="7.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="22.5546875" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="21.88671875" customWidth="1"/>
     <col min="8" max="8" width="20.21875" customWidth="1"/>
     <col min="9" max="9" width="15.5546875" customWidth="1"/>
     <col min="10" max="10" width="14.77734375" customWidth="1"/>
-    <col min="11" max="11" width="35.109375" customWidth="1"/>
+    <col min="11" max="11" width="143.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -516,11 +526,42 @@
       <c r="A2" t="s">
         <v>11</v>
       </c>
+      <c r="B2" s="1">
+        <v>50</v>
+      </c>
+      <c r="C2" s="1">
+        <v>50</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.19689999999999999</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.11799999999999999</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
+      <c r="B3" s="3"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -544,5 +585,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>